<commit_message>
Add footer, jsw-footer blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 12
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-footer.report.xlsx
+++ b/tools/importer/reports/import-jsw-footer.report.xlsx
@@ -139,13 +139,13 @@
     <t>jsw-footer.report.json</t>
   </si>
   <si>
-    <t>["jsw-footer","jsw-footer-links","jsw-footer-social"]</t>
+    <t>["jsw-footer"]</t>
   </si>
   <si>
     <t>jsw-footer</t>
   </si>
   <si>
-    <t>2026-10-27T12:24:51.680Z</t>
+    <t>2026-10-28T09:35:12.831Z</t>
   </si>
   <si>
     <t>JSW Footer</t>

</xml_diff>